<commit_message>
changed oerder of releases columns
</commit_message>
<xml_diff>
--- a/inst/extdata/releases_template.xlsx
+++ b/inst/extdata/releases_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\bio\LobTag2\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5DDD26D-38DF-4FB2-9C10-2EEF381C3C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F63AEBC-2460-4CCD-9E74-12B97503D3E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="releases_template" sheetId="1" r:id="rId1"/>
@@ -936,12 +936,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:W1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="16" max="16" width="11.28515625" customWidth="1"/>
+    <col min="18" max="18" width="11.26171875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -988,13 +988,13 @@
         <v>14</v>
       </c>
       <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
         <v>22</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>15</v>
-      </c>
-      <c r="R1" t="s">
-        <v>16</v>
       </c>
       <c r="S1" t="s">
         <v>17</v>

</xml_diff>